<commit_message>
customer-login page static flow added
</commit_message>
<xml_diff>
--- a/Planning/Shared_Auth_APIs.xlsx
+++ b/Planning/Shared_Auth_APIs.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shubh\Dropbox\PC\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IITB_sem1\cs699_softwareLab\Course_project\Apna-Companion\Planning\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CAFE6CB-ACF1-4268-917E-EF9904C9F6AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Shared auth APIs" sheetId="1" r:id="rId1"/>
@@ -731,7 +731,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -747,7 +747,7 @@
     <col min="12" max="12" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="19">
+    <row r="1" spans="1:12" ht="19.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -768,7 +768,7 @@
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
     </row>
-    <row r="4" spans="1:12" ht="31" customHeight="1">
+    <row r="4" spans="1:12" ht="31.05" customHeight="1">
       <c r="A4" s="4" t="s">
         <v>1</v>
       </c>
@@ -800,7 +800,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="82" customHeight="1">
+    <row r="5" spans="1:12" ht="82.05" customHeight="1">
       <c r="A5" s="5">
         <v>1</v>
       </c>
@@ -864,7 +864,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="152" customHeight="1">
+    <row r="7" spans="1:12" ht="151.94999999999999" customHeight="1">
       <c r="A7" s="5">
         <v>3</v>
       </c>
@@ -928,7 +928,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="82" customHeight="1">
+    <row r="9" spans="1:12" ht="82.05" customHeight="1">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -1032,7 +1032,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F15"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
     <col min="2" max="2" width="54" customWidth="1"/>
@@ -1042,7 +1042,7 @@
     <col min="6" max="6" width="54" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="19">
+    <row r="1" spans="1:6" ht="19.2">
       <c r="A1" s="1" t="s">
         <v>51</v>
       </c>
@@ -1067,7 +1067,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="70" customHeight="1">
+    <row r="4" spans="1:6" ht="70.05" customHeight="1">
       <c r="A4" s="5" t="s">
         <v>58</v>
       </c>
@@ -1087,7 +1087,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="70" customHeight="1">
+    <row r="5" spans="1:6" ht="70.05" customHeight="1">
       <c r="A5" s="12" t="s">
         <v>62</v>
       </c>
@@ -1107,7 +1107,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="70" customHeight="1">
+    <row r="6" spans="1:6" ht="70.05" customHeight="1">
       <c r="A6" s="5" t="s">
         <v>67</v>
       </c>
@@ -1127,7 +1127,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="70" customHeight="1">
+    <row r="7" spans="1:6" ht="70.05" customHeight="1">
       <c r="A7" s="12" t="s">
         <v>71</v>
       </c>
@@ -1147,7 +1147,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="16.5">
+    <row r="10" spans="1:6" ht="16.8">
       <c r="A10" s="13" t="s">
         <v>75</v>
       </c>
@@ -1172,7 +1172,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="55" customHeight="1">
+    <row r="13" spans="1:6" ht="55.05" customHeight="1">
       <c r="A13" s="5" t="s">
         <v>82</v>
       </c>
@@ -1192,7 +1192,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="55" customHeight="1">
+    <row r="14" spans="1:6" ht="55.05" customHeight="1">
       <c r="A14" s="12" t="s">
         <v>88</v>
       </c>
@@ -1212,7 +1212,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="55" customHeight="1">
+    <row r="15" spans="1:6" ht="55.05" customHeight="1">
       <c r="A15" s="5" t="s">
         <v>94</v>
       </c>

</xml_diff>